<commit_message>
deep, stream-curves, staf-web, libs: the Summary band fits one row; a spreadsheet's Preliminary banner is the shorter line
Owner, 2026-10-14. Under a status band the completed workbook's Summary widens column D to 15 (staf_workbook 0.6.1, BANNER_D_W), so the line no longer wraps. Spreadsheets (the calculators' sheets and print headers, and the Summary and ReferenceCurves bands) say Preliminary as 'Reviewed and approved as Preliminary.' (SHEET_NOTES); the app and the PDFs keep the full line. The 16 Preliminary calculators restamped and baked; Draft and Final workbooks are unchanged.
</commit_message>
<xml_diff>
--- a/apps/deep/www/calculators/ak-sqt-adapted.xlsx
+++ b/apps/deep/www/calculators/ak-sqt-adapted.xlsx
@@ -1533,7 +1533,7 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary. Not yet certified for use.</t>
+          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary.</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CB3B"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -1666,7 +1666,7 @@
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary. Not yet certified for use.</t>
+          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary.</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -2728,7 +2728,7 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary. Not yet certified for use.</t>
+          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -5663,7 +5663,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CB3B"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -5707,7 +5707,7 @@
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary. Not yet certified for use.</t>
+          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary.</t>
         </is>
       </c>
     </row>
@@ -8995,7 +8995,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -9029,7 +9029,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary. Not yet certified for use.</t>
+          <t>Assessment status: Preliminary. Reviewed and approved as Preliminary.</t>
         </is>
       </c>
     </row>
@@ -9226,7 +9226,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>
@@ -9682,7 +9682,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CB3B"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary. Not yet certified for use.</oddHeader>
+    <oddHeader>&amp;C&amp;"Calibri,Bold"&amp;KB45309Assessment status: Preliminary._x000a_Reviewed and approved as Preliminary.</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>

</xml_diff>